<commit_message>
Sync from Drive (content + courses.json)
</commit_message>
<xml_diff>
--- a/content/CO0002/CO0002-SOW.xlsx
+++ b/content/CO0002/CO0002-SOW.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="102">
   <si>
     <t>Screen type</t>
   </si>
@@ -40,6 +40,9 @@
   </si>
   <si>
     <t>Introduction to microcontrollers</t>
+  </si>
+  <si>
+    <t>https://i0.wp.com/circuitcellar.com/wp-content/uploads/2016/11/Dobson-Matrix.jpg</t>
   </si>
   <si>
     <t>\CO0002 - Introduction to microcontrollers\media\CO0002 - opening.png</t>
@@ -325,7 +328,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -341,6 +344,11 @@
     <font>
       <sz val="10.0"/>
       <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF467886"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -388,7 +396,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -401,16 +409,19 @@
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -664,13 +675,16 @@
       <c r="D4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>8</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5" s="3">
         <v>0.1</v>
@@ -679,15 +693,15 @@
         <v>6</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="4" t="s">
         <v>11</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" s="3">
         <v>0.1</v>
@@ -696,15 +710,15 @@
         <v>6</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="4" t="s">
         <v>13</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B7" s="3">
         <v>0.1</v>
@@ -713,15 +727,15 @@
         <v>6</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="4" t="s">
         <v>15</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B8" s="3">
         <v>0.1</v>
@@ -730,15 +744,15 @@
         <v>6</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B9" s="3">
         <v>0.1</v>
@@ -749,13 +763,13 @@
       <c r="D9" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>18</v>
+      <c r="E9" s="5" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B10" s="3">
         <v>0.2</v>
@@ -764,15 +778,15 @@
         <v>6</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="5" t="s">
         <v>21</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B11" s="3">
         <v>0.2</v>
@@ -781,15 +795,15 @@
         <v>6</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E11" s="5" t="s">
         <v>23</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12" s="3">
         <v>0.2</v>
@@ -798,15 +812,15 @@
         <v>6</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E12" s="5" t="s">
         <v>26</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B13" s="3">
         <v>0.3</v>
@@ -815,15 +829,15 @@
         <v>6</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E13" s="4" t="s">
         <v>29</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B14" s="3">
         <v>0.3</v>
@@ -832,15 +846,15 @@
         <v>6</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E14" s="4" t="s">
         <v>31</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B15" s="3">
         <v>1.0</v>
@@ -849,15 +863,15 @@
         <v>6</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E15" s="5" t="s">
         <v>33</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B16" s="3">
         <v>1.0</v>
@@ -866,15 +880,15 @@
         <v>6</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="4" t="s">
         <v>36</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B17" s="3">
         <v>1.0</v>
@@ -883,15 +897,15 @@
         <v>6</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E17" s="4" t="s">
         <v>38</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B18" s="3">
         <v>2.0</v>
@@ -900,15 +914,15 @@
         <v>6</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="E18" s="4" t="s">
         <v>40</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B19" s="3">
         <v>2.0</v>
@@ -917,15 +931,15 @@
         <v>6</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E19" s="4" t="s">
         <v>42</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B20" s="3">
         <v>2.0</v>
@@ -934,15 +948,15 @@
         <v>6</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="E20" s="4" t="s">
         <v>44</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B21" s="3">
         <v>2.0</v>
@@ -951,15 +965,15 @@
         <v>6</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E21" s="4" t="s">
         <v>46</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B22" s="3">
         <v>2.0</v>
@@ -968,15 +982,15 @@
         <v>6</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E22" s="4" t="s">
         <v>48</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B23" s="3">
         <v>2.0</v>
@@ -985,15 +999,15 @@
         <v>6</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="E23" s="4" t="s">
         <v>50</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B24" s="3">
         <v>2.0</v>
@@ -1002,15 +1016,15 @@
         <v>6</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E24" s="4" t="s">
         <v>52</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B25" s="3">
         <v>2.0</v>
@@ -1019,15 +1033,15 @@
         <v>6</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="E25" s="4" t="s">
         <v>54</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B26" s="3">
         <v>2.0</v>
@@ -1036,15 +1050,15 @@
         <v>6</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E26" s="4" t="s">
         <v>56</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B27" s="3">
         <v>2.0</v>
@@ -1053,15 +1067,15 @@
         <v>6</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="E27" s="4" t="s">
         <v>58</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B28" s="3">
         <v>2.0</v>
@@ -1070,15 +1084,15 @@
         <v>6</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E28" s="4" t="s">
         <v>60</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B29" s="3">
         <v>2.0</v>
@@ -1087,15 +1101,15 @@
         <v>6</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="E29" s="4" t="s">
         <v>62</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B30" s="3">
         <v>2.0</v>
@@ -1104,15 +1118,15 @@
         <v>6</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="E30" s="4" t="s">
         <v>64</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B31" s="3">
         <v>2.0</v>
@@ -1121,15 +1135,15 @@
         <v>6</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="E31" s="4" t="s">
         <v>66</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B32" s="3">
         <v>2.0</v>
@@ -1138,15 +1152,15 @@
         <v>6</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E32" s="4" t="s">
         <v>68</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B33" s="3">
         <v>2.0</v>
@@ -1155,15 +1169,15 @@
         <v>6</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="E33" s="4" t="s">
         <v>70</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B34" s="3">
         <v>2.0</v>
@@ -1172,15 +1186,15 @@
         <v>6</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="E34" s="4" t="s">
         <v>72</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B35" s="3">
         <v>2.0</v>
@@ -1189,15 +1203,15 @@
         <v>6</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="E35" s="4" t="s">
         <v>74</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B36" s="3">
         <v>2.0</v>
@@ -1206,15 +1220,15 @@
         <v>6</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="E36" s="4" t="s">
         <v>76</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B37" s="3">
         <v>2.0</v>
@@ -1223,15 +1237,15 @@
         <v>6</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="E37" s="4" t="s">
         <v>78</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B38" s="3">
         <v>2.0</v>
@@ -1240,15 +1254,15 @@
         <v>6</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="E38" s="4" t="s">
         <v>80</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B39" s="3">
         <v>2.0</v>
@@ -1257,15 +1271,15 @@
         <v>6</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="E39" s="4" t="s">
         <v>82</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B40" s="3">
         <v>2.0</v>
@@ -1274,15 +1288,15 @@
         <v>6</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="E40" s="4" t="s">
         <v>84</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B41" s="3">
         <v>2.0</v>
@@ -1290,16 +1304,16 @@
       <c r="C41" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D41" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="E41" s="4" t="s">
+      <c r="D41" s="7" t="s">
         <v>86</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B42" s="3">
         <v>2.0</v>
@@ -1307,16 +1321,16 @@
       <c r="C42" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D42" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="E42" s="4" t="s">
+      <c r="D42" s="7" t="s">
         <v>88</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B43" s="3">
         <v>3.0</v>
@@ -1324,16 +1338,16 @@
       <c r="C43" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D43" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="E43" s="4" t="s">
+      <c r="D43" s="7" t="s">
         <v>90</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B44" s="3">
         <v>2.0</v>
@@ -1342,15 +1356,15 @@
         <v>6</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="E44" s="4" t="s">
         <v>92</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B45" s="3">
         <v>4.0</v>
@@ -1358,16 +1372,16 @@
       <c r="C45" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D45" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="E45" s="4" t="s">
+      <c r="D45" s="7" t="s">
         <v>94</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B46" s="3">
         <v>2.0</v>
@@ -1376,15 +1390,15 @@
         <v>6</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="E46" s="4" t="s">
         <v>96</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B47" s="3">
         <v>4.0</v>
@@ -1392,16 +1406,16 @@
       <c r="C47" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D47" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="E47" s="4" t="s">
+      <c r="D47" s="7" t="s">
         <v>98</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B48" s="3">
         <v>30.0</v>
@@ -1410,69 +1424,69 @@
         <v>6</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="E48" s="4" t="s">
         <v>100</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1"/>
     <row r="50" ht="15.75" customHeight="1"/>
     <row r="51" ht="15.75" customHeight="1">
-      <c r="A51" s="7"/>
-      <c r="C51" s="7"/>
-      <c r="D51" s="7"/>
-      <c r="E51" s="7"/>
-      <c r="H51" s="7"/>
+      <c r="A51" s="8"/>
+      <c r="C51" s="8"/>
+      <c r="D51" s="8"/>
+      <c r="E51" s="8"/>
+      <c r="H51" s="8"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="7"/>
-      <c r="B52" s="7"/>
-      <c r="C52" s="7"/>
-      <c r="D52" s="7"/>
-      <c r="G52" s="7"/>
+      <c r="A52" s="8"/>
+      <c r="B52" s="8"/>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
+      <c r="G52" s="8"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="7"/>
-      <c r="B53" s="7"/>
-      <c r="C53" s="7"/>
-      <c r="D53" s="7"/>
-      <c r="G53" s="7"/>
+      <c r="A53" s="8"/>
+      <c r="B53" s="8"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="8"/>
+      <c r="G53" s="8"/>
     </row>
     <row r="54" ht="15.75" customHeight="1">
-      <c r="A54" s="7"/>
-      <c r="C54" s="7"/>
-      <c r="D54" s="7"/>
-      <c r="E54" s="7"/>
-      <c r="H54" s="7"/>
+      <c r="A54" s="8"/>
+      <c r="C54" s="8"/>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8"/>
+      <c r="H54" s="8"/>
     </row>
     <row r="55" ht="15.75" customHeight="1">
-      <c r="A55" s="7"/>
-      <c r="B55" s="7"/>
-      <c r="C55" s="7"/>
-      <c r="D55" s="7"/>
-      <c r="F55" s="7"/>
+      <c r="A55" s="8"/>
+      <c r="B55" s="8"/>
+      <c r="C55" s="8"/>
+      <c r="D55" s="8"/>
+      <c r="F55" s="8"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="7"/>
-      <c r="C56" s="7"/>
-      <c r="D56" s="7"/>
-      <c r="E56" s="7"/>
-      <c r="H56" s="7"/>
+      <c r="A56" s="8"/>
+      <c r="C56" s="8"/>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8"/>
+      <c r="H56" s="8"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="A57" s="7"/>
-      <c r="B57" s="7"/>
-      <c r="C57" s="7"/>
-      <c r="D57" s="7"/>
-      <c r="G57" s="7"/>
+      <c r="A57" s="8"/>
+      <c r="B57" s="8"/>
+      <c r="C57" s="8"/>
+      <c r="D57" s="8"/>
+      <c r="G57" s="8"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="7"/>
-      <c r="C58" s="7"/>
-      <c r="D58" s="7"/>
-      <c r="E58" s="7"/>
-      <c r="H58" s="7"/>
+      <c r="A58" s="8"/>
+      <c r="C58" s="8"/>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8"/>
+      <c r="H58" s="8"/>
     </row>
     <row r="59" ht="15.75" customHeight="1"/>
     <row r="60" ht="15.75" customHeight="1"/>
@@ -2418,14 +2432,15 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="E10"/>
-    <hyperlink r:id="rId2" ref="E11"/>
-    <hyperlink r:id="rId3" ref="E12"/>
-    <hyperlink r:id="rId4" ref="E15"/>
+    <hyperlink r:id="rId1" ref="E4"/>
+    <hyperlink r:id="rId2" ref="E10"/>
+    <hyperlink r:id="rId3" ref="E11"/>
+    <hyperlink r:id="rId4" ref="E12"/>
+    <hyperlink r:id="rId5" ref="E15"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="portrait"/>
-  <drawing r:id="rId5"/>
+  <drawing r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>